<commit_message>
Add company strategy pricing layer
</commit_message>
<xml_diff>
--- a/data/processed/apartment_pricing_recommendations.xlsx
+++ b/data/processed/apartment_pricing_recommendations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC40"/>
+  <dimension ref="A1:AL40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,6 +559,51 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>company_positioning_adjustment_pct</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>sales_phase_adjustment_pct</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>inventory_strategy_adjustment_pct</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>manual_adjustment_pct</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>manual_adjustment_amount</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>strategy_note</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>total_strategy_adjustment_pct</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>final_strategy_price</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>final_strategy_price_per_sqm</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>pricing_status</t>
         </is>
       </c>
@@ -660,7 +705,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>4912343.838260072</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>69383.38754604621</v>
+      </c>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -763,7 +833,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>4466900.325857485</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>68092.99277221777</v>
+      </c>
+      <c r="AL3" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -866,7 +961,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>3501004.232526614</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>61421.12688643183</v>
+      </c>
+      <c r="AL4" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -965,7 +1085,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>4270577.861974038</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>61892.43278223243</v>
+      </c>
+      <c r="AL5" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1068,7 +1213,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>4279135.759502587</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>62016.46028264619</v>
+      </c>
+      <c r="AL6" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1171,7 +1341,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>4270551.626609786</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>61892.05255956212</v>
+      </c>
+      <c r="AL7" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1274,7 +1469,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>6490421.747702251</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>58419.63769308957</v>
+      </c>
+      <c r="AL8" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1377,7 +1597,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>4474290.424801051</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>64844.78876523262</v>
+      </c>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1476,7 +1721,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>4511972.320571836</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>65390.90319669327</v>
+      </c>
+      <c r="AL10" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1579,7 +1849,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>4504797.671148267</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>65286.92277026473</v>
+      </c>
+      <c r="AL11" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1682,7 +1977,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>6709778.606870472</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>60394.0468665209</v>
+      </c>
+      <c r="AL12" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1781,7 +2101,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>4669500.680397624</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>67673.9229043134</v>
+      </c>
+      <c r="AL13" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1880,7 +2225,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>4678058.577926173</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>67797.95040472715</v>
+      </c>
+      <c r="AL14" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -1979,7 +2349,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AC15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>4669474.445033371</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>67673.54268164307</v>
+      </c>
+      <c r="AL15" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2082,7 +2477,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>6889344.566125836</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>62010.30212534506</v>
+      </c>
+      <c r="AL16" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2181,7 +2601,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>4873213.243224635</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>70626.27888731354</v>
+      </c>
+      <c r="AL17" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2284,7 +2729,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>4910895.138995421</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>71172.39331877422</v>
+      </c>
+      <c r="AL18" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2387,7 +2857,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AC19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>4903720.489571851</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>71068.41289234566</v>
+      </c>
+      <c r="AL19" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2490,7 +2985,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AC20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>7108701.425294057</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>63984.7112987764</v>
+      </c>
+      <c r="AL20" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2593,7 +3113,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>5068423.498821209</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>73455.41302639434</v>
+      </c>
+      <c r="AL21" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2692,7 +3237,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AC22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>5076981.396349758</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>73579.44052680809</v>
+      </c>
+      <c r="AL22" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2795,7 +3365,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC23" t="inlineStr">
+      <c r="AC23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>5068397.263456956</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>73455.03280372401</v>
+      </c>
+      <c r="AL23" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -2898,7 +3493,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC24" t="inlineStr">
+      <c r="AC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>7288267.384549422</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>65600.96655760056</v>
+      </c>
+      <c r="AL24" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3001,7 +3621,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC25" t="inlineStr">
+      <c r="AC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>5272136.06164822</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>76407.76900939448</v>
+      </c>
+      <c r="AL25" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3100,7 +3745,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC26" t="inlineStr">
+      <c r="AC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>5309817.957419006</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>76953.88344085516</v>
+      </c>
+      <c r="AL26" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3203,7 +3873,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC27" t="inlineStr">
+      <c r="AC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>5302643.307995436</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>76849.9030144266</v>
+      </c>
+      <c r="AL27" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3306,7 +4001,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC28" t="inlineStr">
+      <c r="AC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>7507624.243717643</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>67575.37573103189</v>
+      </c>
+      <c r="AL28" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3405,7 +4125,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC29" t="inlineStr">
+      <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>5467346.317244794</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>79236.90314847528</v>
+      </c>
+      <c r="AL29" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3504,7 +4249,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC30" t="inlineStr">
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>5475904.214773343</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>79360.93064888903</v>
+      </c>
+      <c r="AL30" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3607,7 +4377,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC31" t="inlineStr">
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>5467320.081880542</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>79236.52292580495</v>
+      </c>
+      <c r="AL31" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3710,7 +4505,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC32" t="inlineStr">
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>7687190.202973006</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>69191.63098985604</v>
+      </c>
+      <c r="AL32" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3809,7 +4629,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC33" t="inlineStr">
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>5671058.880071806</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>82189.25913147544</v>
+      </c>
+      <c r="AL33" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -3908,7 +4753,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC34" t="inlineStr">
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>5708740.775842591</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>82735.3735629361</v>
+      </c>
+      <c r="AL34" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4007,7 +4877,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC35" t="inlineStr">
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>5701566.126419021</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>82631.39313650756</v>
+      </c>
+      <c r="AL35" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4110,7 +5005,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC36" t="inlineStr">
+      <c r="AC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>7906547.062141228</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>71166.04016328738</v>
+      </c>
+      <c r="AL36" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4213,7 +5133,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC37" t="inlineStr">
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>15528580.96488991</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>60848.67149251532</v>
+      </c>
+      <c r="AL37" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4316,7 +5261,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC38" t="inlineStr">
+      <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>15781094.02076194</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>60673.17962615124</v>
+      </c>
+      <c r="AL38" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4419,7 +5389,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC39" t="inlineStr">
+      <c r="AC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>11285398.3930051</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>66345.66956499177</v>
+      </c>
+      <c r="AL39" t="inlineStr">
         <is>
           <t>priced</t>
         </is>
@@ -4518,7 +5513,32 @@
           <t>synthetic_poc</t>
         </is>
       </c>
-      <c r="AC40" t="inlineStr">
+      <c r="AC40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>10543870.66979108</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>66480.89955732079</v>
+      </c>
+      <c r="AL40" t="inlineStr">
         <is>
           <t>priced</t>
         </is>

</xml_diff>

<commit_message>
Update pricing weights to 70/30 historical/current market blend
</commit_message>
<xml_diff>
--- a/data/processed/apartment_pricing_recommendations.xlsx
+++ b/data/processed/apartment_pricing_recommendations.xlsx
@@ -673,22 +673,22 @@
         <v>116351.1520137065</v>
       </c>
       <c r="T2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V2" t="n">
-        <v>2141759.780352378</v>
+        <v>2998463.692493329</v>
       </c>
       <c r="W2" t="n">
-        <v>4118830.781285209</v>
+        <v>2471298.468771125</v>
       </c>
       <c r="X2" t="n">
-        <v>6260590.561637588</v>
+        <v>5469762.161264455</v>
       </c>
       <c r="Y2" t="n">
-        <v>88426.42036211283</v>
+        <v>77256.52770147535</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -725,10 +725,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ2" t="n">
-        <v>6135378.750404836</v>
+        <v>5360366.918039165</v>
       </c>
       <c r="AK2" t="n">
-        <v>86657.89195487056</v>
+        <v>75711.39714744584</v>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
@@ -801,22 +801,22 @@
         <v>109347.8552969606</v>
       </c>
       <c r="T3" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V3" t="n">
-        <v>1978650.80768399</v>
+        <v>2770111.130757586</v>
       </c>
       <c r="W3" t="n">
-        <v>3586609.653740306</v>
+        <v>2151965.792244183</v>
       </c>
       <c r="X3" t="n">
-        <v>5565260.461424297</v>
+        <v>4922076.92300177</v>
       </c>
       <c r="Y3" t="n">
-        <v>84836.28752171184</v>
+        <v>75031.66041161235</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -853,10 +853,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ3" t="n">
-        <v>5453955.252195811</v>
+        <v>4823635.384541734</v>
       </c>
       <c r="AK3" t="n">
-        <v>83139.56177127761</v>
+        <v>73531.0272033801</v>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
@@ -929,22 +929,22 @@
         <v>88508.23686668056</v>
       </c>
       <c r="T4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U4" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V4" t="n">
-        <v>1697776.238037175</v>
+        <v>2376886.733252045</v>
       </c>
       <c r="W4" t="n">
-        <v>2522484.750700396</v>
+        <v>1513490.850420238</v>
       </c>
       <c r="X4" t="n">
-        <v>4220260.988737571</v>
+        <v>3890377.583672282</v>
       </c>
       <c r="Y4" t="n">
-        <v>74039.6664690802</v>
+        <v>68252.23831004003</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -981,10 +981,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4135855.76896282</v>
+        <v>3812570.031998836</v>
       </c>
       <c r="AK4" t="n">
-        <v>72558.87313969858</v>
+        <v>66887.19354383924</v>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
@@ -1053,22 +1053,22 @@
         <v>81115.30850722632</v>
       </c>
       <c r="T5" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U5" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V5" t="n">
-        <v>2168796.217093366</v>
+        <v>3036314.703930712</v>
       </c>
       <c r="W5" t="n">
-        <v>2798478.143499308</v>
+        <v>1679086.886099585</v>
       </c>
       <c r="X5" t="n">
-        <v>4967274.360592674</v>
+        <v>4715401.590030297</v>
       </c>
       <c r="Y5" t="n">
-        <v>71989.48348685035</v>
+        <v>68339.15347869995</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1105,10 +1105,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ5" t="n">
-        <v>4867928.873380821</v>
+        <v>4621093.55822969</v>
       </c>
       <c r="AK5" t="n">
-        <v>70549.69381711335</v>
+        <v>66972.37040912594</v>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
@@ -1181,22 +1181,22 @@
         <v>81528.7335086055</v>
       </c>
       <c r="T6" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V6" t="n">
-        <v>2168796.217093366</v>
+        <v>3036314.703930712</v>
       </c>
       <c r="W6" t="n">
-        <v>2812741.30604689</v>
+        <v>1687644.783628134</v>
       </c>
       <c r="X6" t="n">
-        <v>4981537.523140255</v>
+        <v>4723959.487558845</v>
       </c>
       <c r="Y6" t="n">
-        <v>72196.19598753993</v>
+        <v>68463.18097911371</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1233,10 +1233,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ6" t="n">
-        <v>4881906.77267745</v>
+        <v>4629480.297807668</v>
       </c>
       <c r="AK6" t="n">
-        <v>70752.27206778913</v>
+        <v>67093.91735953142</v>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
@@ -1309,22 +1309,22 @@
         <v>81114.04109832525</v>
       </c>
       <c r="T7" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V7" t="n">
-        <v>2168796.217093366</v>
+        <v>3036314.703930712</v>
       </c>
       <c r="W7" t="n">
-        <v>2798434.417892221</v>
+        <v>1679060.650735333</v>
       </c>
       <c r="X7" t="n">
-        <v>4967230.634985587</v>
+        <v>4715375.354666045</v>
       </c>
       <c r="Y7" t="n">
-        <v>71988.8497823998</v>
+        <v>68338.77325602964</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1361,10 +1361,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ7" t="n">
-        <v>4867886.022285875</v>
+        <v>4621067.847572724</v>
       </c>
       <c r="AK7" t="n">
-        <v>70549.07278675181</v>
+        <v>66971.99779090905</v>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
@@ -1437,22 +1437,22 @@
         <v>79214.26887609315</v>
       </c>
       <c r="T8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U8" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V8" t="n">
-        <v>3511586.398587545</v>
+        <v>4916220.958022563</v>
       </c>
       <c r="W8" t="n">
-        <v>4400352.636066974</v>
+        <v>2640211.581640184</v>
       </c>
       <c r="X8" t="n">
-        <v>7911939.03465452</v>
+        <v>7556432.539662747</v>
       </c>
       <c r="Y8" t="n">
-        <v>71214.5727691676</v>
+        <v>68014.69432639737</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1489,10 +1489,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ8" t="n">
-        <v>7753700.253961429</v>
+        <v>7405303.888869491</v>
       </c>
       <c r="AK8" t="n">
-        <v>69790.28131378425</v>
+        <v>66654.40043986941</v>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
@@ -1565,22 +1565,22 @@
         <v>81579.71457299804</v>
       </c>
       <c r="T9" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U9" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V9" t="n">
-        <v>2252293.452065718</v>
+        <v>3153210.832892005</v>
       </c>
       <c r="W9" t="n">
-        <v>2814500.152768433</v>
+        <v>1688700.09166106</v>
       </c>
       <c r="X9" t="n">
-        <v>5066793.604834151</v>
+        <v>4841910.924553065</v>
       </c>
       <c r="Y9" t="n">
-        <v>73431.79137440799</v>
+        <v>70172.62209497196</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1617,10 +1617,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ9" t="n">
-        <v>4965457.732737468</v>
+        <v>4745072.706062003</v>
       </c>
       <c r="AK9" t="n">
-        <v>71963.15554691982</v>
+        <v>68769.1696530725</v>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
@@ -1689,22 +1689,22 @@
         <v>83400.09601120026</v>
       </c>
       <c r="T10" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U10" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V10" t="n">
-        <v>2252293.452065718</v>
+        <v>3153210.832892005</v>
       </c>
       <c r="W10" t="n">
-        <v>2877303.312386409</v>
+        <v>1726381.987431846</v>
       </c>
       <c r="X10" t="n">
-        <v>5129596.764452128</v>
+        <v>4879592.820323851</v>
       </c>
       <c r="Y10" t="n">
-        <v>74341.9820935091</v>
+        <v>70718.73652643262</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1741,10 +1741,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ10" t="n">
-        <v>5027004.829163085</v>
+        <v>4782000.963917374</v>
       </c>
       <c r="AK10" t="n">
-        <v>72855.14245163891</v>
+        <v>69304.36179590397</v>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
@@ -1817,22 +1817,22 @@
         <v>83053.49458977176</v>
       </c>
       <c r="T11" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U11" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V11" t="n">
-        <v>2252293.452065718</v>
+        <v>3153210.832892005</v>
       </c>
       <c r="W11" t="n">
-        <v>2865345.563347125</v>
+        <v>1719207.338008275</v>
       </c>
       <c r="X11" t="n">
-        <v>5117639.015412844</v>
+        <v>4872418.170900281</v>
       </c>
       <c r="Y11" t="n">
-        <v>74168.68138279484</v>
+        <v>70614.75610000407</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1869,10 +1869,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ11" t="n">
-        <v>5015286.235104587</v>
+        <v>4774969.807482275</v>
       </c>
       <c r="AK11" t="n">
-        <v>72685.30775513894</v>
+        <v>69202.46097800399</v>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
@@ -1945,22 +1945,22 @@
         <v>79972.06971325737</v>
       </c>
       <c r="T12" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V12" t="n">
-        <v>3595083.633559898</v>
+        <v>5033117.086983857</v>
       </c>
       <c r="W12" t="n">
-        <v>4442448.472571447</v>
+        <v>2665469.083542868</v>
       </c>
       <c r="X12" t="n">
-        <v>8037532.106131345</v>
+        <v>7698586.170526724</v>
       </c>
       <c r="Y12" t="n">
-        <v>72345.02345752786</v>
+        <v>69294.20495523604</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1997,10 +1997,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ12" t="n">
-        <v>7876781.464008718</v>
+        <v>7544614.44711619</v>
       </c>
       <c r="AK12" t="n">
-        <v>70898.1229883773</v>
+        <v>67908.32085613132</v>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
@@ -2069,22 +2069,22 @@
         <v>81633.38115903844</v>
       </c>
       <c r="T13" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U13" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V13" t="n">
-        <v>2335790.687038071</v>
+        <v>3270106.961853298</v>
       </c>
       <c r="W13" t="n">
-        <v>2816351.649986826</v>
+        <v>1689810.989992096</v>
       </c>
       <c r="X13" t="n">
-        <v>5152142.337024897</v>
+        <v>4959917.951845394</v>
       </c>
       <c r="Y13" t="n">
-        <v>74668.72952209997</v>
+        <v>71882.86886732456</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2121,10 +2121,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ13" t="n">
-        <v>5049099.490284399</v>
+        <v>4860719.592808487</v>
       </c>
       <c r="AK13" t="n">
-        <v>73175.35493165796</v>
+        <v>70445.21148997807</v>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
@@ -2193,22 +2193,22 @@
         <v>82046.80616041762</v>
       </c>
       <c r="T14" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U14" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V14" t="n">
-        <v>2335790.687038071</v>
+        <v>3270106.961853298</v>
       </c>
       <c r="W14" t="n">
-        <v>2830614.812534408</v>
+        <v>1698368.887520645</v>
       </c>
       <c r="X14" t="n">
-        <v>5166405.499572478</v>
+        <v>4968475.849373943</v>
       </c>
       <c r="Y14" t="n">
-        <v>74875.44202278955</v>
+        <v>72006.8963677383</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2245,10 +2245,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ14" t="n">
-        <v>5063077.389581028</v>
+        <v>4869106.332386464</v>
       </c>
       <c r="AK14" t="n">
-        <v>73377.93318233374</v>
+        <v>70566.75844038354</v>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
@@ -2317,22 +2317,22 @@
         <v>81632.11375013737</v>
       </c>
       <c r="T15" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U15" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V15" t="n">
-        <v>2335790.687038071</v>
+        <v>3270106.961853298</v>
       </c>
       <c r="W15" t="n">
-        <v>2816307.924379739</v>
+        <v>1689784.754627844</v>
       </c>
       <c r="X15" t="n">
-        <v>5152098.61141781</v>
+        <v>4959891.716481142</v>
       </c>
       <c r="Y15" t="n">
-        <v>74668.09581764942</v>
+        <v>71882.48864465422</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2369,10 +2369,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ15" t="n">
-        <v>5049056.639189453</v>
+        <v>4860693.882151519</v>
       </c>
       <c r="AK15" t="n">
-        <v>73174.73390129642</v>
+        <v>70444.83887176114</v>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
@@ -2445,22 +2445,22 @@
         <v>79536.02416839769</v>
       </c>
       <c r="T16" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U16" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V16" t="n">
-        <v>3678580.86853225</v>
+        <v>5150013.21594515</v>
       </c>
       <c r="W16" t="n">
-        <v>4418226.142554492</v>
+        <v>2650935.685532695</v>
       </c>
       <c r="X16" t="n">
-        <v>8096807.011086741</v>
+        <v>7800948.901477845</v>
       </c>
       <c r="Y16" t="n">
-        <v>72878.55095487616</v>
+        <v>70215.56166946756</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2497,10 +2497,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ16" t="n">
-        <v>7934870.870865007</v>
+        <v>7644929.923448288</v>
       </c>
       <c r="AK16" t="n">
-        <v>71420.97993577864</v>
+        <v>68811.2504360782</v>
       </c>
       <c r="AL16" t="inlineStr">
         <is>
@@ -2569,22 +2569,22 @@
         <v>82097.78722481016</v>
       </c>
       <c r="T17" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U17" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V17" t="n">
-        <v>2419287.922010423</v>
+        <v>3387003.090814592</v>
       </c>
       <c r="W17" t="n">
-        <v>2832373.659255951</v>
+        <v>1699424.19555357</v>
       </c>
       <c r="X17" t="n">
-        <v>5251661.581266373</v>
+        <v>5086427.286368162</v>
       </c>
       <c r="Y17" t="n">
-        <v>76111.03740965758</v>
+        <v>73716.33748359655</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2621,10 +2621,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ17" t="n">
-        <v>5146628.349641046</v>
+        <v>4984698.740640799</v>
       </c>
       <c r="AK17" t="n">
-        <v>74588.81666146443</v>
+        <v>72242.01073392462</v>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
@@ -2697,22 +2697,22 @@
         <v>83918.16866301239</v>
       </c>
       <c r="T18" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U18" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V18" t="n">
-        <v>2419287.922010423</v>
+        <v>3387003.090814592</v>
       </c>
       <c r="W18" t="n">
-        <v>2895176.818873927</v>
+        <v>1737106.091324356</v>
       </c>
       <c r="X18" t="n">
-        <v>5314464.740884351</v>
+        <v>5124109.182138949</v>
       </c>
       <c r="Y18" t="n">
-        <v>77021.22812875871</v>
+        <v>74262.45191505723</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2749,10 +2749,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ18" t="n">
-        <v>5208175.446066664</v>
+        <v>5021626.998496169</v>
       </c>
       <c r="AK18" t="n">
-        <v>75480.80356618353</v>
+        <v>72777.20287675607</v>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
@@ -2825,22 +2825,22 @@
         <v>83571.56724158386</v>
       </c>
       <c r="T19" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U19" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V19" t="n">
-        <v>2419287.922010423</v>
+        <v>3387003.090814592</v>
       </c>
       <c r="W19" t="n">
-        <v>2883219.069834644</v>
+        <v>1729931.441900786</v>
       </c>
       <c r="X19" t="n">
-        <v>5302506.991845067</v>
+        <v>5116934.532715378</v>
       </c>
       <c r="Y19" t="n">
-        <v>76847.92741804445</v>
+        <v>74158.47148862867</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2877,10 +2877,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ19" t="n">
-        <v>5196456.852008165</v>
+        <v>5014595.842061071</v>
       </c>
       <c r="AK19" t="n">
-        <v>75310.96886968355</v>
+        <v>72675.30205885609</v>
       </c>
       <c r="AL19" t="inlineStr">
         <is>
@@ -2953,22 +2953,22 @@
         <v>80293.82500556191</v>
       </c>
       <c r="T20" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U20" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V20" t="n">
-        <v>3762078.103504602</v>
+        <v>5266909.344906443</v>
       </c>
       <c r="W20" t="n">
-        <v>4460321.979058964</v>
+        <v>2676193.187435378</v>
       </c>
       <c r="X20" t="n">
-        <v>8222400.082563566</v>
+        <v>7943102.532341821</v>
       </c>
       <c r="Y20" t="n">
-        <v>74009.00164323642</v>
+        <v>71495.07229830623</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -3005,10 +3005,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ20" t="n">
-        <v>8057952.080912295</v>
+        <v>7784240.481694984</v>
       </c>
       <c r="AK20" t="n">
-        <v>72528.8216103717</v>
+        <v>70065.1708523401</v>
       </c>
       <c r="AL20" t="inlineStr">
         <is>
@@ -3081,22 +3081,22 @@
         <v>82151.45381085057</v>
       </c>
       <c r="T21" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U21" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V21" t="n">
-        <v>2502785.156982775</v>
+        <v>3503899.219775885</v>
       </c>
       <c r="W21" t="n">
-        <v>2834225.156474344</v>
+        <v>1700535.093884607</v>
       </c>
       <c r="X21" t="n">
-        <v>5337010.31345712</v>
+        <v>5204434.313660492</v>
       </c>
       <c r="Y21" t="n">
-        <v>77347.97555734956</v>
+        <v>75426.58425594916</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3133,10 +3133,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ21" t="n">
-        <v>5230270.107187978</v>
+        <v>5100345.627387282</v>
       </c>
       <c r="AK21" t="n">
-        <v>75801.01604620258</v>
+        <v>73918.05257083019</v>
       </c>
       <c r="AL21" t="inlineStr">
         <is>
@@ -3205,22 +3205,22 @@
         <v>82564.87881222973</v>
       </c>
       <c r="T22" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U22" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V22" t="n">
-        <v>2502785.156982775</v>
+        <v>3503899.219775885</v>
       </c>
       <c r="W22" t="n">
-        <v>2848488.319021926</v>
+        <v>1709092.991413155</v>
       </c>
       <c r="X22" t="n">
-        <v>5351273.476004701</v>
+        <v>5212992.211189041</v>
       </c>
       <c r="Y22" t="n">
-        <v>77554.68805803914</v>
+        <v>75550.61175636291</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3257,10 +3257,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ22" t="n">
-        <v>5244248.006484607</v>
+        <v>5108732.36696526</v>
       </c>
       <c r="AK22" t="n">
-        <v>76003.59429687836</v>
+        <v>74039.59952123565</v>
       </c>
       <c r="AL22" t="inlineStr">
         <is>
@@ -3333,22 +3333,22 @@
         <v>82150.1864019495</v>
       </c>
       <c r="T23" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U23" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V23" t="n">
-        <v>2502785.156982775</v>
+        <v>3503899.219775885</v>
       </c>
       <c r="W23" t="n">
-        <v>2834181.430867258</v>
+        <v>1700508.858520354</v>
       </c>
       <c r="X23" t="n">
-        <v>5336966.587850032</v>
+        <v>5204408.078296239</v>
       </c>
       <c r="Y23" t="n">
-        <v>77347.34185289902</v>
+        <v>75426.20403327883</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3385,10 +3385,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ23" t="n">
-        <v>5230227.256093032</v>
+        <v>5100319.916730314</v>
       </c>
       <c r="AK23" t="n">
-        <v>75800.39501584104</v>
+        <v>73917.67995261325</v>
       </c>
       <c r="AL23" t="inlineStr">
         <is>
@@ -3461,22 +3461,22 @@
         <v>79857.77946070227</v>
       </c>
       <c r="T24" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U24" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V24" t="n">
-        <v>3845575.338476955</v>
+        <v>5383805.473867737</v>
       </c>
       <c r="W24" t="n">
-        <v>4436099.64904201</v>
+        <v>2661659.789425206</v>
       </c>
       <c r="X24" t="n">
-        <v>8281674.987518965</v>
+        <v>8045465.263292942</v>
       </c>
       <c r="Y24" t="n">
-        <v>74542.52914058475</v>
+        <v>72416.42901253773</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ24" t="n">
-        <v>8116041.487768586</v>
+        <v>7884555.958027083</v>
       </c>
       <c r="AK24" t="n">
-        <v>73051.67855777305</v>
+        <v>70968.10043228698</v>
       </c>
       <c r="AL24" t="inlineStr">
         <is>
@@ -3589,22 +3589,22 @@
         <v>82615.85987662229</v>
       </c>
       <c r="T25" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U25" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V25" t="n">
-        <v>2586282.391955127</v>
+        <v>3620795.348737178</v>
       </c>
       <c r="W25" t="n">
-        <v>2850247.165743469</v>
+        <v>1710148.299446081</v>
       </c>
       <c r="X25" t="n">
-        <v>5436529.557698596</v>
+        <v>5330943.64818326</v>
       </c>
       <c r="Y25" t="n">
-        <v>78790.2834449072</v>
+        <v>77260.05287222116</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3641,10 +3641,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ25" t="n">
-        <v>5327798.966544624</v>
+        <v>5224324.775219595</v>
       </c>
       <c r="AK25" t="n">
-        <v>77214.47777600905</v>
+        <v>75714.85181477675</v>
       </c>
       <c r="AL25" t="inlineStr">
         <is>
@@ -3713,22 +3713,22 @@
         <v>84436.24131482451</v>
       </c>
       <c r="T26" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U26" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V26" t="n">
-        <v>2586282.391955127</v>
+        <v>3620795.348737178</v>
       </c>
       <c r="W26" t="n">
-        <v>2913050.325361446</v>
+        <v>1747830.195216867</v>
       </c>
       <c r="X26" t="n">
-        <v>5499332.717316573</v>
+        <v>5368625.543954046</v>
       </c>
       <c r="Y26" t="n">
-        <v>79700.47416400831</v>
+        <v>77806.16730368182</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3765,10 +3765,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ26" t="n">
-        <v>5389346.062970242</v>
+        <v>5261253.033074965</v>
       </c>
       <c r="AK26" t="n">
-        <v>78106.46468072814</v>
+        <v>76250.04395760818</v>
       </c>
       <c r="AL26" t="inlineStr">
         <is>
@@ -3841,22 +3841,22 @@
         <v>84089.63989339599</v>
       </c>
       <c r="T27" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U27" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V27" t="n">
-        <v>2586282.391955127</v>
+        <v>3620795.348737178</v>
       </c>
       <c r="W27" t="n">
-        <v>2901092.576322162</v>
+        <v>1740655.545793297</v>
       </c>
       <c r="X27" t="n">
-        <v>5487374.968277289</v>
+        <v>5361450.894530475</v>
       </c>
       <c r="Y27" t="n">
-        <v>79527.17345329403</v>
+        <v>77702.18687725326</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3893,10 +3893,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ27" t="n">
-        <v>5377627.468911743</v>
+        <v>5254221.876639865</v>
       </c>
       <c r="AK27" t="n">
-        <v>77936.62998422816</v>
+        <v>76148.14313970819</v>
       </c>
       <c r="AL27" t="inlineStr">
         <is>
@@ -3969,22 +3969,22 @@
         <v>80615.58029786649</v>
       </c>
       <c r="T28" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U28" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V28" t="n">
-        <v>3929072.573449307</v>
+        <v>5500701.60282903</v>
       </c>
       <c r="W28" t="n">
-        <v>4478195.485546483</v>
+        <v>2686917.29132789</v>
       </c>
       <c r="X28" t="n">
-        <v>8407268.058995791</v>
+        <v>8187618.89415692</v>
       </c>
       <c r="Y28" t="n">
-        <v>75672.97982894501</v>
+        <v>73695.93964137642</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -4021,10 +4021,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ28" t="n">
-        <v>8239122.697815875</v>
+        <v>8023866.516273782</v>
       </c>
       <c r="AK28" t="n">
-        <v>74159.52023236611</v>
+        <v>72222.0208485489</v>
       </c>
       <c r="AL28" t="inlineStr">
         <is>
@@ -4093,22 +4093,22 @@
         <v>82669.52646266269</v>
       </c>
       <c r="T29" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U29" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V29" t="n">
-        <v>2669779.62692748</v>
+        <v>3737691.477698471</v>
       </c>
       <c r="W29" t="n">
-        <v>2852098.662961863</v>
+        <v>1711259.197777117</v>
       </c>
       <c r="X29" t="n">
-        <v>5521878.289889342</v>
+        <v>5448950.675475589</v>
       </c>
       <c r="Y29" t="n">
-        <v>80027.22159259916</v>
+        <v>78970.29964457375</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
@@ -4145,10 +4145,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ29" t="n">
-        <v>5411440.724091555</v>
+        <v>5339971.661966077</v>
       </c>
       <c r="AK29" t="n">
-        <v>78426.67716074717</v>
+        <v>77390.89365168227</v>
       </c>
       <c r="AL29" t="inlineStr">
         <is>
@@ -4217,22 +4217,22 @@
         <v>83082.95146404185</v>
       </c>
       <c r="T30" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U30" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V30" t="n">
-        <v>2669779.62692748</v>
+        <v>3737691.477698471</v>
       </c>
       <c r="W30" t="n">
-        <v>2866361.825509444</v>
+        <v>1719817.095305666</v>
       </c>
       <c r="X30" t="n">
-        <v>5536141.452436924</v>
+        <v>5457508.573004138</v>
       </c>
       <c r="Y30" t="n">
-        <v>80233.93409328876</v>
+        <v>79094.3271449875</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4269,10 +4269,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ30" t="n">
-        <v>5425418.623388185</v>
+        <v>5348358.401544055</v>
       </c>
       <c r="AK30" t="n">
-        <v>78629.25541142297</v>
+        <v>77512.44060208775</v>
       </c>
       <c r="AL30" t="inlineStr">
         <is>
@@ -4345,22 +4345,22 @@
         <v>82668.25905376161</v>
       </c>
       <c r="T31" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U31" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V31" t="n">
-        <v>2669779.62692748</v>
+        <v>3737691.477698471</v>
       </c>
       <c r="W31" t="n">
-        <v>2852054.937354776</v>
+        <v>1711232.962412865</v>
       </c>
       <c r="X31" t="n">
-        <v>5521834.564282255</v>
+        <v>5448924.440111337</v>
       </c>
       <c r="Y31" t="n">
-        <v>80026.58788814863</v>
+        <v>78969.91942190344</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -4397,10 +4397,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ31" t="n">
-        <v>5411397.87299661</v>
+        <v>5339945.95130911</v>
       </c>
       <c r="AK31" t="n">
-        <v>78426.05613038565</v>
+        <v>77390.52103346537</v>
       </c>
       <c r="AL31" t="inlineStr">
         <is>
@@ -4473,22 +4473,22 @@
         <v>80179.53475300681</v>
       </c>
       <c r="T32" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U32" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V32" t="n">
-        <v>4012569.808421659</v>
+        <v>5617597.731790323</v>
       </c>
       <c r="W32" t="n">
-        <v>4453973.155529528</v>
+        <v>2672383.893317717</v>
       </c>
       <c r="X32" t="n">
-        <v>8466542.963951187</v>
+        <v>8289981.625108039</v>
       </c>
       <c r="Y32" t="n">
-        <v>76206.50732629331</v>
+        <v>74617.29635560792</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4525,10 +4525,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ32" t="n">
-        <v>8297212.104672164</v>
+        <v>8124181.992605878</v>
       </c>
       <c r="AK32" t="n">
-        <v>74682.37717976746</v>
+        <v>73124.95042849575</v>
       </c>
       <c r="AL32" t="inlineStr">
         <is>
@@ -4597,22 +4597,22 @@
         <v>83133.93252843441</v>
       </c>
       <c r="T33" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U33" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V33" t="n">
-        <v>2753276.861899832</v>
+        <v>3854587.606659765</v>
       </c>
       <c r="W33" t="n">
-        <v>2868120.672230987</v>
+        <v>1720872.403338592</v>
       </c>
       <c r="X33" t="n">
-        <v>5621397.534130819</v>
+        <v>5575460.009998357</v>
       </c>
       <c r="Y33" t="n">
-        <v>81469.52948015679</v>
+        <v>80803.76826084575</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
@@ -4649,10 +4649,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ33" t="n">
-        <v>5508969.583448202</v>
+        <v>5463950.80979839</v>
       </c>
       <c r="AK33" t="n">
-        <v>79840.13889055366</v>
+        <v>79187.69289562883</v>
       </c>
       <c r="AL33" t="inlineStr">
         <is>
@@ -4721,22 +4721,22 @@
         <v>84954.31396663663</v>
       </c>
       <c r="T34" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U34" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V34" t="n">
-        <v>2753276.861899832</v>
+        <v>3854587.606659765</v>
       </c>
       <c r="W34" t="n">
-        <v>2930923.831848964</v>
+        <v>1758554.299109378</v>
       </c>
       <c r="X34" t="n">
-        <v>5684200.693748796</v>
+        <v>5613141.905769143</v>
       </c>
       <c r="Y34" t="n">
-        <v>82379.72019925792</v>
+        <v>81349.88269230642</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4773,10 +4773,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ34" t="n">
-        <v>5570516.67987382</v>
+        <v>5500879.06765376</v>
       </c>
       <c r="AK34" t="n">
-        <v>80732.12579527276</v>
+        <v>79722.8850384603</v>
       </c>
       <c r="AL34" t="inlineStr">
         <is>
@@ -4845,22 +4845,22 @@
         <v>84607.71254520811</v>
       </c>
       <c r="T35" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U35" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V35" t="n">
-        <v>2753276.861899832</v>
+        <v>3854587.606659765</v>
       </c>
       <c r="W35" t="n">
-        <v>2918966.08280968</v>
+        <v>1751379.649685808</v>
       </c>
       <c r="X35" t="n">
-        <v>5672242.944709511</v>
+        <v>5605967.256345573</v>
       </c>
       <c r="Y35" t="n">
-        <v>82206.41948854364</v>
+        <v>81245.90226587787</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4897,10 +4897,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ35" t="n">
-        <v>5558798.085815321</v>
+        <v>5493847.911218661</v>
       </c>
       <c r="AK35" t="n">
-        <v>80562.29109877277</v>
+        <v>79620.98422056031</v>
       </c>
       <c r="AL35" t="inlineStr">
         <is>
@@ -4973,22 +4973,22 @@
         <v>80937.33559017103</v>
       </c>
       <c r="T36" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U36" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V36" t="n">
-        <v>4096067.043394012</v>
+        <v>5734493.860751617</v>
       </c>
       <c r="W36" t="n">
-        <v>4496068.992034</v>
+        <v>2697641.3952204</v>
       </c>
       <c r="X36" t="n">
-        <v>8592136.035428012</v>
+        <v>8432135.255972017</v>
       </c>
       <c r="Y36" t="n">
-        <v>77336.95801465357</v>
+        <v>75896.80698444659</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -5025,10 +5025,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ36" t="n">
-        <v>8420293.314719452</v>
+        <v>8263492.550852576</v>
       </c>
       <c r="AK36" t="n">
-        <v>75790.2188543605</v>
+        <v>74378.87084475766</v>
       </c>
       <c r="AL36" t="inlineStr">
         <is>
@@ -5101,22 +5101,22 @@
         <v>85057.43771268504</v>
       </c>
       <c r="T37" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U37" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V37" t="n">
-        <v>8710682.27042982</v>
+        <v>12194955.17860175</v>
       </c>
       <c r="W37" t="n">
-        <v>10853329.05213861</v>
+        <v>6511997.431283167</v>
       </c>
       <c r="X37" t="n">
-        <v>19564011.32256843</v>
+        <v>18706952.60988491</v>
       </c>
       <c r="Y37" t="n">
-        <v>76661.48637370075</v>
+        <v>73303.10583810703</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -5153,10 +5153,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ37" t="n">
-        <v>19172731.09611706</v>
+        <v>18332813.55768722</v>
       </c>
       <c r="AK37" t="n">
-        <v>75128.25664622674</v>
+        <v>71837.04372134489</v>
       </c>
       <c r="AL37" t="inlineStr">
         <is>
@@ -5229,22 +5229,22 @@
         <v>85168.20807928006</v>
       </c>
       <c r="T38" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U38" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V38" t="n">
-        <v>8864381.110059649</v>
+        <v>12410133.55408351</v>
       </c>
       <c r="W38" t="n">
-        <v>11076125.46071037</v>
+        <v>6645675.276426223</v>
       </c>
       <c r="X38" t="n">
-        <v>19940506.57077002</v>
+        <v>19055808.83050973</v>
       </c>
       <c r="Y38" t="n">
-        <v>76664.76959158023</v>
+        <v>73263.3941965003</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -5281,10 +5281,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ38" t="n">
-        <v>19541696.43935462</v>
+        <v>18674692.65389954</v>
       </c>
       <c r="AK38" t="n">
-        <v>75131.47419974863</v>
+        <v>71798.1263125703</v>
       </c>
       <c r="AL38" t="inlineStr">
         <is>
@@ -5357,22 +5357,22 @@
         <v>82575.22951274294</v>
       </c>
       <c r="T39" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U39" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V39" t="n">
-        <v>6052458.621032804</v>
+        <v>8473442.069445925</v>
       </c>
       <c r="W39" t="n">
-        <v>7023023.270058786</v>
+        <v>4213813.962035271</v>
       </c>
       <c r="X39" t="n">
-        <v>13075481.89109159</v>
+        <v>12687256.0314812</v>
       </c>
       <c r="Y39" t="n">
-        <v>76869.38207578831</v>
+        <v>74587.04310100643</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -5409,10 +5409,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ39" t="n">
-        <v>12813972.25326976</v>
+        <v>12433510.91085157</v>
       </c>
       <c r="AK39" t="n">
-        <v>75331.99443427254</v>
+        <v>73095.30223898632</v>
       </c>
       <c r="AL39" t="inlineStr">
         <is>
@@ -5481,22 +5481,22 @@
         <v>83835.47003044009</v>
       </c>
       <c r="T40" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="U40" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="V40" t="n">
-        <v>5669502.009471828</v>
+        <v>7937302.813260559</v>
       </c>
       <c r="W40" t="n">
-        <v>6648152.773413899</v>
+        <v>3988891.664048339</v>
       </c>
       <c r="X40" t="n">
-        <v>12317654.78288573</v>
+        <v>11926194.4773089</v>
       </c>
       <c r="Y40" t="n">
-        <v>77664.9103586742</v>
+        <v>75196.68648996785</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -5533,10 +5533,10 @@
         <v>-0.02</v>
       </c>
       <c r="AJ40" t="n">
-        <v>12071301.68722801</v>
+        <v>11687670.58776272</v>
       </c>
       <c r="AK40" t="n">
-        <v>76111.6121515007</v>
+        <v>73692.75276016849</v>
       </c>
       <c r="AL40" t="inlineStr">
         <is>

</xml_diff>